<commit_message>
Make Meridian Ops visibly demo-ready for the challenge
- Refresh demo fixtures with rule-triggering tickets (R1 winter BS6, R2 hill,
  R4 Vertex gate, R6 Orion year, R8 beyond-50km, R11 new-driver night)
- Mixed Hindi-English maintenance notes for realistic parsing surface
- Improve context Q&A: answers "why was vehicle X rejected?" with real reasons
- Visual pipeline stages on RUN (ingest → … → approval gate)
- Fix run_pipeline --fresh for /tmp state
- Rewrite README with clear judge demo flow and scoring-aligned checklist
</commit_message>
<xml_diff>
--- a/maintenance_log.xlsx
+++ b/maintenance_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Brake pads replaced. Service due on 2026-02-15</t>
+          <t>Brake pads change kiya. Service due on 2026-02-15. Temporary jugaad still on suspension.</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Temporary jugaad on suspension. Brake work done</t>
+          <t>Engine heater not working. Brake work last month. Hill route ke liye not safe.</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Engine heater not functional. Service overdue</t>
+          <t>Service overdue. Full service due on 2025-12-01. Temporary repair on clutch.</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Full service completed. Brake inspection OK</t>
+          <t>Full service completed. Brakes OK. Engine heater working.</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Routine check. No issues</t>
+          <t>Routine check. Koi issue nahi.</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,30 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Service due on 2026-09-01. All good</t>
+          <t>Service due on 2026-09-01. All systems normal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DL01OP0123</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>55000</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Cold chain unit check. Refrigeration OK for Orion loads.</t>
         </is>
       </c>
     </row>

</xml_diff>